<commit_message>
because of persnickety rich and els
</commit_message>
<xml_diff>
--- a/rules/CORE-002050/negative/01/data/CORE-002050-negative-01.xlsx
+++ b/rules/CORE-002050/negative/01/data/CORE-002050-negative-01.xlsx
@@ -36,11 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -57,7 +53,16 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -69,8 +74,13 @@
       <name val="Calibri"/>
       <color rgb="FF000000"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -84,6 +94,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -113,7 +135,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -122,6 +144,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,18 +480,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="2" t="str">
         <v>Product</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="2" t="str">
         <v>Version</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="2" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="2" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -483,18 +507,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="3" t="str">
         <v>Filename</v>
       </c>
-      <c r="B1" s="4" t="str">
+      <c r="B1" s="3" t="str">
         <v>Label</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="2" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="2" t="str">
         <v>Trial Summary</v>
       </c>
     </row>
@@ -510,103 +534,103 @@
   <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="4" t="str">
         <v>Error group</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="4" t="str">
         <v>Sheet</v>
       </c>
-      <c r="C1" s="3" t="str">
+      <c r="C1" s="4" t="str">
         <v>Error level</v>
       </c>
-      <c r="D1" s="3" t="str">
+      <c r="D1" s="4" t="str">
         <v>Row num</v>
       </c>
-      <c r="E1" s="3" t="str">
+      <c r="E1" s="4" t="str">
         <v>Variable</v>
       </c>
-      <c r="F1" s="3" t="str">
+      <c r="F1" s="4" t="str">
         <v>Error value</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="4" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C2" s="3" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="str">
+      <c r="E2" s="4" t="str">
         <v>TSPARMCD</v>
       </c>
-      <c r="F2" s="3" t="str">
-        <v>FDATCHSP</v>
+      <c r="F2" s="4" t="str">
+        <v>CTAUG</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="str">
+      <c r="B3" s="4" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C3" s="3" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="str">
+      <c r="E3" s="4" t="str">
         <v>TSVAL</v>
       </c>
       <c r="F3" s="5" t="str">
-        <v>Study Data Technical Conformance Guide v4.2.0</v>
+        <v>Influenza Therapeutic Area User Guide v1.0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="str">
+      <c r="B4" s="4" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C4" s="3" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="4">
         <v>6</v>
       </c>
-      <c r="E4" s="3" t="str">
+      <c r="E4" s="4" t="str">
         <v>TSPARMCD</v>
       </c>
-      <c r="F4" s="3" t="str">
-        <v>FDATCHSP</v>
+      <c r="F4" s="4" t="str">
+        <v>CTAUG</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="str">
+      <c r="B5" s="4" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C5" s="3" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="4">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="str">
+      <c r="E5" s="4" t="str">
         <v>TSVAL</v>
       </c>
       <c r="F5" s="5" t="str">
-        <v>Fake Guide Doc</v>
+        <v>Dyslipidemia Therapeutic Area User Guide v1</v>
       </c>
     </row>
   </sheetData>
@@ -621,37 +645,37 @@
   <dimension ref="A1:K6"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="3" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="4" t="str">
+      <c r="B1" s="3" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="C1" s="4" t="str">
+      <c r="C1" s="3" t="str">
         <v>TSSEQ</v>
       </c>
-      <c r="D1" s="4" t="str">
+      <c r="D1" s="3" t="str">
         <v>TSGRPID</v>
       </c>
-      <c r="E1" s="4" t="str">
+      <c r="E1" s="3" t="str">
         <v>TSPARMCD</v>
       </c>
-      <c r="F1" s="4" t="str">
+      <c r="F1" s="3" t="str">
         <v>TSPARM</v>
       </c>
-      <c r="G1" s="4" t="str">
+      <c r="G1" s="3" t="str">
         <v>TSVAL</v>
       </c>
-      <c r="H1" s="4" t="str">
+      <c r="H1" s="3" t="str">
         <v>TSVALNF</v>
       </c>
-      <c r="I1" s="4" t="str">
+      <c r="I1" s="3" t="str">
         <v>TSVALCD</v>
       </c>
-      <c r="J1" s="4" t="str">
+      <c r="J1" s="3" t="str">
         <v>TSVCDREF</v>
       </c>
-      <c r="K1" s="4" t="str">
+      <c r="K1" s="3" t="str">
         <v>TSVCDVER</v>
       </c>
     </row>
@@ -659,104 +683,104 @@
       <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="7" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="7" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="7" t="str">
         <v>Group ID</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="7" t="str">
         <v>Trial Summary Parameter Short Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="7" t="str">
         <v>Trial Summary Parameter</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="7" t="str">
         <v>Parameter Value</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="7" t="str">
         <v>Parameter Null Flavor</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="7" t="str">
         <v>Parameter Value Code</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="7" t="str">
         <v>Name of the Reference Terminology</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="7" t="str">
         <v>Version of the Reference Terminology</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
+      <c r="A3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="7" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="str">
+      <c r="A4" s="7" t="str">
         <v>12</v>
       </c>
-      <c r="B4" s="6" t="str">
+      <c r="B4" s="7" t="str">
         <v>2</v>
       </c>
-      <c r="C4" s="6" t="str">
+      <c r="C4" s="7" t="str">
         <v>8</v>
       </c>
-      <c r="D4" s="6" t="str">
+      <c r="D4" s="7" t="str">
         <v>8</v>
       </c>
-      <c r="E4" s="6" t="str">
+      <c r="E4" s="7" t="str">
         <v>8</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F4" s="7" t="str">
         <v>40</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="7" t="str">
         <v>194</v>
       </c>
-      <c r="H4" s="6" t="str">
+      <c r="H4" s="7" t="str">
         <v>3</v>
       </c>
-      <c r="I4" s="6" t="str">
+      <c r="I4" s="7" t="str">
         <v>11</v>
       </c>
-      <c r="J4" s="6" t="str">
+      <c r="J4" s="7" t="str">
         <v>9</v>
       </c>
-      <c r="K4" s="6" t="str">
+      <c r="K4" s="7" t="str">
         <v>10</v>
       </c>
     </row>
@@ -773,14 +797,14 @@
       <c r="D5" s="5" t="str">
         <v/>
       </c>
-      <c r="E5" s="7" t="str">
-        <v>FDATCHSP</v>
+      <c r="E5" s="8" t="str">
+        <v>CTAUG</v>
       </c>
       <c r="F5" s="5" t="str">
-        <v>FDA Technical Specification Response</v>
-      </c>
-      <c r="G5" s="7" t="str">
-        <v>Study Data Technical Conformance Guide v4.2.0</v>
+        <v>CDISC Therapeutic Area User Guide</v>
+      </c>
+      <c r="G5" s="9" t="str">
+        <v>Influenza Therapeutic Area User Guide v1.0</v>
       </c>
       <c r="H5" s="5" t="str">
         <v>NA</v>
@@ -792,7 +816,7 @@
         <v/>
       </c>
       <c r="K5" s="5" t="str">
-        <v>2025-03-28</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -808,14 +832,14 @@
       <c r="D6" s="5" t="str">
         <v/>
       </c>
-      <c r="E6" s="7" t="str">
-        <v>FDATCHSP</v>
+      <c r="E6" s="9" t="str">
+        <v>CTAUG</v>
       </c>
       <c r="F6" s="5" t="str">
-        <v>FDA Technical Specification Response</v>
-      </c>
-      <c r="G6" s="7" t="str">
-        <v>Fake Guide Doc</v>
+        <v>CDISC Therapeutic Area User Guide</v>
+      </c>
+      <c r="G6" s="9" t="str">
+        <v>Dyslipidemia Therapeutic Area User Guide v1</v>
       </c>
       <c r="H6" s="5" t="str">
         <v>NA</v>
@@ -827,7 +851,7 @@
         <v/>
       </c>
       <c r="K6" s="5" t="str">
-        <v>2025-03-28</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>